<commit_message>
Update seating.xlsx for FEHD August 4
Sync the workbook to the FEHD list updated August 4: add TALES and mark IRON COW TAIWANESE BEEF NOODLE as delisted.
</commit_message>
<xml_diff>
--- a/seating.xlsx
+++ b/seating.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meta" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seating'!$A$1:$F$980</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seating'!$A$1:$F$981</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
@@ -72,7 +72,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -94,6 +94,11 @@
         <fgColor rgb="FFFFF3C4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3C4"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -107,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -128,6 +133,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -493,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F980"/>
+  <dimension ref="A1:F981"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.875" defaultRowHeight="15"/>
   <cols>
     <col width="13.98828125" customWidth="1" min="1" max="1"/>
@@ -28644,10 +28650,38 @@
       </c>
       <c r="F980" s="4" t="n"/>
     </row>
+    <row r="981">
+      <c r="A981" s="7" t="inlineStr">
+        <is>
+          <t>3198801431</t>
+        </is>
+      </c>
+      <c r="B981" s="8" t="inlineStr">
+        <is>
+          <t>TALES</t>
+        </is>
+      </c>
+      <c r="C981" s="8" t="inlineStr">
+        <is>
+          <t>TALES</t>
+        </is>
+      </c>
+      <c r="D981" s="8" t="inlineStr">
+        <is>
+          <t>Sai Kung</t>
+        </is>
+      </c>
+      <c r="E981" s="8" t="inlineStr">
+        <is>
+          <t>G/F, 36 SEE CHEUNG STREET, SAI KUNG, NEW TERRITORIES</t>
+        </is>
+      </c>
+      <c r="F981" s="14" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F980"/>
+  <autoFilter ref="A1:F981"/>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F980" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Please choose indoor or outdoor (or clear the cell)." promptTitle="Seating" prompt="Choose indoor or outdoor, or leave blank if unknown." type="list">
+    <dataValidation sqref="F2:F981" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Please choose indoor or outdoor (or clear the cell)." promptTitle="Seating" prompt="Choose indoor or outdoor, or leave blank if unknown." type="list">
       <formula1>"indoor,outdoor"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Set PizzaExpress seating to indoor
Update licence 2297809166 in seating.xlsx.
</commit_message>
<xml_diff>
--- a/seating.xlsx
+++ b/seating.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martintan/Documents/GitHub/paws-plates-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D0BFD02-B4A3-A848-9032-2CB1EF34EF1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C61D21A-D3A8-F942-8AD5-EFC65A64723A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19060" yWindow="1200" windowWidth="25680" windowHeight="22920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5117" uniqueCount="3155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5118" uniqueCount="3155">
   <si>
     <t>FEHD Licence</t>
   </si>
@@ -18309,7 +18309,9 @@
       <c r="E457" s="3" t="s">
         <v>1493</v>
       </c>
-      <c r="F457" s="4"/>
+      <c r="F457" s="4" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="458" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A458" s="2" t="s">

</xml_diff>

<commit_message>
Mark 麵聖 seating as indoor
Set FEHD licence 2252810613 to indoor seating.
</commit_message>
<xml_diff>
--- a/seating.xlsx
+++ b/seating.xlsx
@@ -14387,7 +14387,9 @@
       <c r="E244" s="3" t="s">
         <v>798</v>
       </c>
-      <c r="F244" s="4"/>
+      <c r="F244" s="4" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="245" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A245" s="2" t="s">

</xml_diff>

<commit_message>
Sync seating.xlsx with FEHD August 6
Add 2.0 CAFE AND BAR (2252810491); no delisted licences.
</commit_message>
<xml_diff>
--- a/seating.xlsx
+++ b/seating.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5118" uniqueCount="3155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5123" uniqueCount="3160">
   <si>
     <t>FEHD Licence</t>
   </si>
@@ -9490,6 +9490,21 @@
   </si>
   <si>
     <t>nothing is downloaded and nothing is changed.</t>
+  </si>
+  <si>
+    <t>2252810491</t>
+  </si>
+  <si>
+    <t>2.0 CAFE AND BAR</t>
+  </si>
+  <si>
+    <t>PORTION A OF SHOP NO. S201, 2/F, KAI TAK CRUISE TERMINAL, 33 SHING FUNG ROAD, KOWLOON</t>
+  </si>
+  <si>
+    <t>August 6</t>
+  </si>
+  <si>
+    <t>2026-08-06 19:10</t>
   </si>
 </sst>
 </file>
@@ -9912,7 +9927,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F983"/>
+  <dimension ref="A1:F984"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -27971,10 +27986,28 @@
         <v>47</v>
       </c>
     </row>
+    <row r="984" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A984" s="2" t="s">
+        <v>3155</v>
+      </c>
+      <c r="B984" s="3" t="s">
+        <v>3156</v>
+      </c>
+      <c r="C984" s="3" t="s">
+        <v>3156</v>
+      </c>
+      <c r="D984" s="3" t="s">
+        <v>600</v>
+      </c>
+      <c r="E984" s="3" t="s">
+        <v>3157</v>
+      </c>
+      <c r="F984" s="4"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F981" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:F984" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" errorTitle="Invalid value" error="Please choose indoor or outdoor (or clear the cell)." promptTitle="Seating" prompt="Choose indoor or outdoor, or leave blank if unknown." sqref="F2:F981" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" errorTitle="Invalid value" error="Please choose indoor or outdoor (or clear the cell)." promptTitle="Seating" prompt="Choose indoor or outdoor, or leave blank if unknown." sqref="F2:F984" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"indoor,outdoor"</formula1>
     </dataValidation>
   </dataValidations>
@@ -28085,7 +28118,7 @@
         <v>3144</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>3145</v>
+        <v>3158</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -28101,7 +28134,7 @@
         <v>3148</v>
       </c>
       <c r="B3" s="13">
-        <v>979</v>
+        <v>983</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -28109,7 +28142,7 @@
         <v>3149</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>3150</v>
+        <v>3159</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
update seating arrangement based on top 10 list
</commit_message>
<xml_diff>
--- a/seating.xlsx
+++ b/seating.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="19060" yWindow="1200" windowWidth="25680" windowHeight="22920" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Seating" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="READ ME" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Meta" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seating" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="READ ME" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meta" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seating'!$A$1:$F$985</definedName>
@@ -5782,7 +5782,11 @@
           <t>SHOP NO.1404, 14/F, TOWER II, THE TWINS, 12 MUK CHUI STREET, KAI TAK, KOWLOON</t>
         </is>
       </c>
-      <c r="F185" s="4" t="n"/>
+      <c r="F185" s="4" t="inlineStr">
+        <is>
+          <t>indoor</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
@@ -7382,7 +7386,11 @@
           <t>SHOP NO. G002, G/F, AIRSIDE, 2 CONCORDE ROAD, KAI TAK, KOWLOON</t>
         </is>
       </c>
-      <c r="F240" s="4" t="n"/>
+      <c r="F240" s="4" t="inlineStr">
+        <is>
+          <t>indoor</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
@@ -7838,7 +7846,11 @@
           <t>SHOP 212A, 2/F, MARITIME SQUARE 1, 31-33 TSING KING ROAD, TSING YI, NEW TERRITORIES</t>
         </is>
       </c>
-      <c r="F256" s="4" t="n"/>
+      <c r="F256" s="4" t="inlineStr">
+        <is>
+          <t>indoor</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
@@ -8066,7 +8078,11 @@
           <t>SEATING AREA A, B AND UNIT 10, LEVEL 11, MEGABOX, ENTERPRISE SQUARE FIVE, 38 WANG CHIU ROAD, KOWLOON BAY, KOWLOON</t>
         </is>
       </c>
-      <c r="F264" s="4" t="n"/>
+      <c r="F264" s="4" t="inlineStr">
+        <is>
+          <t>indoor</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
@@ -25430,7 +25446,11 @@
           <t>2/F (PORTION), REGAL KOWLOON HOTEL, 71 MODY ROAD, TSIM SHA TSUI EAST, KOWLOON</t>
         </is>
       </c>
-      <c r="F866" s="4" t="n"/>
+      <c r="F866" s="4" t="inlineStr">
+        <is>
+          <t>indoor</t>
+        </is>
+      </c>
     </row>
     <row r="867">
       <c r="A867" s="2" t="inlineStr">
@@ -26970,7 +26990,11 @@
           <t>SHOPS NO. B141-B142, LEVEL1, YOHO MIX, 1 LONG LOK ROAD, YUEN LONG, NEW TERRITORIES</t>
         </is>
       </c>
-      <c r="F920" s="4" t="n"/>
+      <c r="F920" s="4" t="inlineStr">
+        <is>
+          <t>indoor</t>
+        </is>
+      </c>
     </row>
     <row r="921">
       <c r="A921" s="2" t="inlineStr">
@@ -27790,7 +27814,11 @@
           <t>G/F, LOTS 153 (PART) AND 154 S.A (PART) IN D.D. 102, WING PING TSUEN, SAN TIN, YUEN LONG, NEW TERRITORIES</t>
         </is>
       </c>
-      <c r="F949" s="4" t="n"/>
+      <c r="F949" s="4" t="inlineStr">
+        <is>
+          <t>indoor</t>
+        </is>
+      </c>
     </row>
     <row r="950">
       <c r="A950" s="2" t="inlineStr">

</xml_diff>

<commit_message>
FEHD sync August 11: 2 added, 0 delisted
+ [2215801915] Zola Beach Bar / Zola Beach Bar (Southern)
+ [3161808504] HARU / 旭宵食堂 (Yau Tsim)
</commit_message>
<xml_diff>
--- a/seating.xlsx
+++ b/seating.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Delisted" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seating'!$A$1:$F$985</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seating'!$A$1:$F$987</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F985"/>
+  <dimension ref="A1:F987"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28852,10 +28852,66 @@
       </c>
       <c r="F985" s="16" t="inlineStr"/>
     </row>
+    <row r="986">
+      <c r="A986" s="7" t="inlineStr">
+        <is>
+          <t>2215801915</t>
+        </is>
+      </c>
+      <c r="B986" s="8" t="inlineStr">
+        <is>
+          <t>Zola Beach Bar</t>
+        </is>
+      </c>
+      <c r="C986" s="8" t="inlineStr">
+        <is>
+          <t>Zola Beach Bar</t>
+        </is>
+      </c>
+      <c r="D986" s="8" t="inlineStr">
+        <is>
+          <t>Southern</t>
+        </is>
+      </c>
+      <c r="E986" s="8" t="inlineStr">
+        <is>
+          <t>SHOP NO. 2 AND OUTSIDE SEATING ACCOMMODATION AT SHOP FRONT, G/F., NO. 90 STANLEY MAIN STREET, STANLEY, HONG KONG</t>
+        </is>
+      </c>
+      <c r="F986" s="16" t="inlineStr"/>
+    </row>
+    <row r="987">
+      <c r="A987" s="7" t="inlineStr">
+        <is>
+          <t>3161808504</t>
+        </is>
+      </c>
+      <c r="B987" s="8" t="inlineStr">
+        <is>
+          <t>HARU</t>
+        </is>
+      </c>
+      <c r="C987" s="8" t="inlineStr">
+        <is>
+          <t>旭宵食堂</t>
+        </is>
+      </c>
+      <c r="D987" s="8" t="inlineStr">
+        <is>
+          <t>Yau Tsim</t>
+        </is>
+      </c>
+      <c r="E987" s="8" t="inlineStr">
+        <is>
+          <t>AREA NO.4 AT ART PARK, WEST KOWLOON CULTURAL DISTRICT, KOWLOON</t>
+        </is>
+      </c>
+      <c r="F987" s="16" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F985"/>
+  <autoFilter ref="A1:F987"/>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F985" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F987" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"indoor,outdoor"</formula1>
     </dataValidation>
   </dataValidations>
@@ -29005,7 +29061,7 @@
       </c>
       <c r="B1" s="12" t="inlineStr">
         <is>
-          <t>August 10</t>
+          <t>August 11</t>
         </is>
       </c>
     </row>
@@ -29028,7 +29084,7 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>984</v>
+        <v>986</v>
       </c>
     </row>
     <row r="4">
@@ -29039,7 +29095,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>2026-08-10 15:29</t>
+          <t>2026-08-11 16:04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
FEHD sync August 12: 1 added, 0 delisted
+ [2261824223] HTIKE EASY / 泰簡 (Yau Tsim)
</commit_message>
<xml_diff>
--- a/seating.xlsx
+++ b/seating.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Delisted" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seating'!$A$1:$F$987</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seating'!$A$1:$F$988</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F987"/>
+  <dimension ref="A1:F988"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28908,10 +28908,38 @@
       </c>
       <c r="F987" s="16" t="inlineStr"/>
     </row>
+    <row r="988">
+      <c r="A988" s="7" t="inlineStr">
+        <is>
+          <t>2261824223</t>
+        </is>
+      </c>
+      <c r="B988" s="8" t="inlineStr">
+        <is>
+          <t>HTIKE EASY</t>
+        </is>
+      </c>
+      <c r="C988" s="8" t="inlineStr">
+        <is>
+          <t>泰簡</t>
+        </is>
+      </c>
+      <c r="D988" s="8" t="inlineStr">
+        <is>
+          <t>Yau Tsim</t>
+        </is>
+      </c>
+      <c r="E988" s="8" t="inlineStr">
+        <is>
+          <t>SHOP 5, G/F, PO FAT BUILDING, NOS. 273-285 TEMPLE STREET, KOWLOON</t>
+        </is>
+      </c>
+      <c r="F988" s="16" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F987"/>
+  <autoFilter ref="A1:F988"/>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F987" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F988" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"indoor,outdoor"</formula1>
     </dataValidation>
   </dataValidations>
@@ -29061,7 +29089,7 @@
       </c>
       <c r="B1" s="12" t="inlineStr">
         <is>
-          <t>August 11</t>
+          <t>August 12</t>
         </is>
       </c>
     </row>
@@ -29084,7 +29112,7 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>986</v>
+        <v>987</v>
       </c>
     </row>
     <row r="4">
@@ -29095,7 +29123,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>2026-08-11 16:04</t>
+          <t>2026-08-12 16:09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
FEHD sync August 19: 3 added, 0 delisted
+ [3197802312] Moon Ocean / Moon Ocean (Sha Tin)
+ [2263809071] URBAN Cafe / URBAN Cafe (Sham Shui Po)
+ [3194803299] MASAM / MASAM (Yuen Long)
</commit_message>
<xml_diff>
--- a/seating.xlsx
+++ b/seating.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Delisted" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seating'!$A$1:$F$988</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seating'!$A$1:$F$991</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -533,7 +533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F988"/>
+  <dimension ref="A1:F991"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28960,10 +28960,94 @@
       </c>
       <c r="F988" s="20" t="inlineStr"/>
     </row>
+    <row r="989">
+      <c r="A989" s="18" t="inlineStr">
+        <is>
+          <t>3197802312</t>
+        </is>
+      </c>
+      <c r="B989" s="19" t="inlineStr">
+        <is>
+          <t>Moon Ocean</t>
+        </is>
+      </c>
+      <c r="C989" s="19" t="inlineStr">
+        <is>
+          <t>Moon Ocean</t>
+        </is>
+      </c>
+      <c r="D989" s="19" t="inlineStr">
+        <is>
+          <t>Sha Tin</t>
+        </is>
+      </c>
+      <c r="E989" s="19" t="inlineStr">
+        <is>
+          <t>SHOP A, G/F &amp; COCKLOFT, HING WAN HOUSE, 74-76 CHIK CHUEN STREET, TAI WAI, SHA TIN, NEW TERRITORIES</t>
+        </is>
+      </c>
+      <c r="F989" s="20" t="inlineStr"/>
+    </row>
+    <row r="990">
+      <c r="A990" s="18" t="inlineStr">
+        <is>
+          <t>2263809071</t>
+        </is>
+      </c>
+      <c r="B990" s="19" t="inlineStr">
+        <is>
+          <t>URBAN Cafe</t>
+        </is>
+      </c>
+      <c r="C990" s="19" t="inlineStr">
+        <is>
+          <t>URBAN Cafe</t>
+        </is>
+      </c>
+      <c r="D990" s="19" t="inlineStr">
+        <is>
+          <t>Sham Shui Po</t>
+        </is>
+      </c>
+      <c r="E990" s="19" t="inlineStr">
+        <is>
+          <t>PORTION A OF UNIT 103, 1/F, LAI SUN COMMERCIAL CENTRE, 680 CHEUNG SHA WAN ROAD, LAI CHI KOK, KOWLOON</t>
+        </is>
+      </c>
+      <c r="F990" s="20" t="inlineStr"/>
+    </row>
+    <row r="991">
+      <c r="A991" s="18" t="inlineStr">
+        <is>
+          <t>3194803299</t>
+        </is>
+      </c>
+      <c r="B991" s="19" t="inlineStr">
+        <is>
+          <t>MASAM</t>
+        </is>
+      </c>
+      <c r="C991" s="19" t="inlineStr">
+        <is>
+          <t>MASAM</t>
+        </is>
+      </c>
+      <c r="D991" s="19" t="inlineStr">
+        <is>
+          <t>Yuen Long</t>
+        </is>
+      </c>
+      <c r="E991" s="19" t="inlineStr">
+        <is>
+          <t>SHOP D, G/F, LEE FAT HOUSE, NO. 5 YAN LOK SQUARE, YUEN LONG, NEW TERRITORIES</t>
+        </is>
+      </c>
+      <c r="F991" s="20" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F988"/>
+  <autoFilter ref="A1:F991"/>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F988" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F991" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"indoor,outdoor"</formula1>
     </dataValidation>
   </dataValidations>
@@ -29113,7 +29197,7 @@
       </c>
       <c r="B1" s="12" t="inlineStr">
         <is>
-          <t>August 18</t>
+          <t>August 19</t>
         </is>
       </c>
     </row>
@@ -29136,7 +29220,7 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>987</v>
+        <v>990</v>
       </c>
     </row>
     <row r="4">
@@ -29147,7 +29231,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>2026-08-18 15:30</t>
+          <t>2026-08-19 15:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
FEHD sync August 20: 1 added, 0 delisted
+ [3118809361] For Single / For Single (Central/Western)
</commit_message>
<xml_diff>
--- a/seating.xlsx
+++ b/seating.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Delisted" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seating'!$A$1:$F$991</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seating'!$A$1:$F$992</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -533,7 +533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F991"/>
+  <dimension ref="A1:F992"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29044,10 +29044,38 @@
       </c>
       <c r="F991" s="20" t="inlineStr"/>
     </row>
+    <row r="992">
+      <c r="A992" s="18" t="inlineStr">
+        <is>
+          <t>3118809361</t>
+        </is>
+      </c>
+      <c r="B992" s="19" t="inlineStr">
+        <is>
+          <t>For Single</t>
+        </is>
+      </c>
+      <c r="C992" s="19" t="inlineStr">
+        <is>
+          <t>For Single</t>
+        </is>
+      </c>
+      <c r="D992" s="19" t="inlineStr">
+        <is>
+          <t>Central/Western</t>
+        </is>
+      </c>
+      <c r="E992" s="19" t="inlineStr">
+        <is>
+          <t>SHOP D, G/F., FULL HARVEST BUILDING, 6-18 HAU WO STREET, HONG KONG</t>
+        </is>
+      </c>
+      <c r="F992" s="20" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F991"/>
+  <autoFilter ref="A1:F992"/>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F991" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F992" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"indoor,outdoor"</formula1>
     </dataValidation>
   </dataValidations>
@@ -29197,7 +29225,7 @@
       </c>
       <c r="B1" s="12" t="inlineStr">
         <is>
-          <t>August 19</t>
+          <t>August 20</t>
         </is>
       </c>
     </row>
@@ -29220,7 +29248,7 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>990</v>
+        <v>991</v>
       </c>
     </row>
     <row r="4">
@@ -29231,7 +29259,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>2026-08-19 15:30</t>
+          <t>2026-08-20 15:33</t>
         </is>
       </c>
     </row>

</xml_diff>